<commit_message>
latest amendments for PreProd
</commit_message>
<xml_diff>
--- a/DFC.App.ExploreCareers.UI.FunctionalTests/Data/JobProfiles.xlsx
+++ b/DFC.App.ExploreCareers.UI.FunctionalTests/Data/JobProfiles.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25330"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\ESFAAutomation\dfc-app-explorecareers\DFC.App.ExploreCareers.UI.FunctionalTests\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF0F1B8-AC6D-44A4-A30C-558A1EE8E4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8FE5DA0-52B2-4A5F-8548-AAAE96288B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -152,9 +152,6 @@
     <t xml:space="preserve"> Law and legal                     </t>
   </si>
   <si>
-    <t xml:space="preserve"> Barristers' clerk                                             </t>
-  </si>
-  <si>
     <t xml:space="preserve"> Immigration adviser (non-government)                          </t>
   </si>
   <si>
@@ -183,6 +180,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Train conductor                                               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barrister's clerk                      </t>
   </si>
 </sst>
 </file>
@@ -766,7 +766,7 @@
         <v>771</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C24" t="s">
         <v>34</v>
@@ -777,7 +777,7 @@
         <v>783</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C25" t="s">
         <v>34</v>
@@ -788,10 +788,10 @@
         <v>831</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -799,10 +799,10 @@
         <v>891</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -810,10 +810,10 @@
         <v>956</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -821,10 +821,10 @@
         <v>965</v>
       </c>
       <c r="B29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -832,10 +832,10 @@
         <v>968</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C30" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>